<commit_message>
Enllaç a la política de privacitat de l'Ajuntament; Naturpunt sense activitat
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012ateu6UxL7MVs9JrFhHhY1
</commit_message>
<xml_diff>
--- a/dades.xlsx
+++ b/dades.xlsx
@@ -980,7 +980,11 @@
           <t>Política de privacitat (enllaç)</t>
         </is>
       </c>
-      <c r="B9" s="4" t="inlineStr"/>
+      <c r="B9" s="4" t="inlineStr">
+        <is>
+          <t>https://www.lalqueriadasnar.es/aviso-legal/politica-privacidad/</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -4651,11 +4655,7 @@
           <t>Naturpunt, SL</t>
         </is>
       </c>
-      <c r="C9" s="4" t="inlineStr">
-        <is>
-          <t>Activitat per confirmar</t>
-        </is>
-      </c>
+      <c r="C9" s="4" t="inlineStr"/>
       <c r="D9" s="4" t="n"/>
       <c r="E9" s="4" t="n"/>
     </row>

</xml_diff>

<commit_message>
Agència Impuls: calendari 2026 verificat
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012ateu6UxL7MVs9JrFhHhY1
</commit_message>
<xml_diff>
--- a/dades.xlsx
+++ b/dades.xlsx
@@ -2538,7 +2538,7 @@
           <t>Consultes individuals gratuïtes d'una hora, aproximadament
 Model de negoci, màrqueting i gestió econòmica i financera
 Cerca d'ajudes i posada en marxa
-Sessions a Cocentaina en 2026: 5 de novembre i 9 de desembre (9.30–14 h)</t>
+Pròximes sessions a Cocentaina: dijous 5 de novembre i dimecres 9 de desembre de 2026, de 9.30 a 14 h</t>
         </is>
       </c>
       <c r="K7" s="4" t="inlineStr">
@@ -2579,17 +2579,13 @@
       </c>
       <c r="W7" s="4" t="inlineStr">
         <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="X7" s="4" t="inlineStr">
-        <is>
-          <t>Pendent: confirmar calendari</t>
-        </is>
-      </c>
+          <t>sí</t>
+        </is>
+      </c>
+      <c r="X7" s="4" t="inlineStr"/>
       <c r="Y7" s="4" t="inlineStr">
         <is>
-          <t>Convocatòria Agència Impuls 2026, EmprenemJunts [F29].</t>
+          <t>Agenda 2026 de l'Agència Impuls, EmprenemJunts [F29]. Consulta: 26/10/2026.</t>
         </is>
       </c>
       <c r="Z7" s="4" t="inlineStr">

</xml_diff>

<commit_message>
Nau històrica del Bambú: data d'inauguració i primer ús
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012ateu6UxL7MVs9JrFhHhY1
</commit_message>
<xml_diff>
--- a/dades.xlsx
+++ b/dades.xlsx
@@ -3463,7 +3463,8 @@
       <c r="J16" s="4" t="inlineStr">
         <is>
           <t>Usos previstos: culturals i formatius
-Rehabilitació parcial contractada el 2023; recuperació presentada el juny de 2024
+Rehabilitació parcial contractada el 2023 i inaugurada l'11 de juny de 2024
+Primer ús: exposició del 30é aniversari de la Colla Dimonis Rafolins
 Col·laboració entre l'Ajuntament i Hinojosa Paper</t>
         </is>
       </c>
@@ -3519,7 +3520,7 @@
       </c>
       <c r="Y16" s="4" t="inlineStr">
         <is>
-          <t>TVA, rehabilitació de l'antiga nau del Bambú [F21].</t>
+          <t>TVA, 22/06/2024, rehabilitació de l'antiga nau del Bambú [F21].</t>
         </is>
       </c>
       <c r="Z16" s="4" t="inlineStr">

</xml_diff>

<commit_message>
Obrir una activitat: enllaços als tràmits de la seu electrònica
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012ateu6UxL7MVs9JrFhHhY1
</commit_message>
<xml_diff>
--- a/dades.xlsx
+++ b/dades.xlsx
@@ -2103,7 +2103,7 @@
       </c>
       <c r="K3" s="4" t="inlineStr">
         <is>
-          <t>Registre presencial de l'Ajuntament o seu electrònica.</t>
+          <t>Presentació electrònica a la seu de l'Ajuntament (amb certificat digital o Cl@ve) o al registre presencial. Si no saps quin tràmit et correspon, consulta-ho abans a l'Ajuntament.</t>
         </is>
       </c>
       <c r="L3" s="4" t="inlineStr">
@@ -2134,7 +2134,10 @@
       </c>
       <c r="R3" s="4" t="inlineStr">
         <is>
-          <t>Sol·licituds i impresos | https://www.lalqueriadasnar.es/el-ayuntamiento/solicitudes-e-impresos/
+          <t>Botiga, oficina, despatx o taller: declaració responsable o comunicació d'activitat | https://lalqueriadasnar.sedelectronica.es/catalog/t/df2d1685-af1d-454c-90dd-f0d077868573
+Bar, cafeteria o restaurant: declaració responsable d'establiments públics | https://lalqueriadasnar.sedelectronica.es/catalog/t/36fa4d83-67b8-4671-808c-09185dae1c62
+Activitat amb més impacte ambiental: sol·licitud de llicència d'activitat | https://lalqueriadasnar.sedelectronica.es/catalog/t/bf5e9be9-4ba9-4bbd-86cd-2f915f8b3c78
+Establiment públic que requereix llicència | https://lalqueriadasnar.sedelectronica.es/catalog/t/87679048-b42c-47a7-8c33-3d54d162f988
 Ordenances municipals | https://www.lalqueriadasnar.es/el-ayuntamiento/ordenanzas-y-actas-de-plenos/</t>
         </is>
       </c>
@@ -2157,7 +2160,7 @@
       </c>
       <c r="X3" s="4" t="inlineStr">
         <is>
-          <t>Pendent: taxes i model d'obertura</t>
+          <t>Pendent: taxes</t>
         </is>
       </c>
       <c r="Y3" s="4" t="inlineStr">

</xml_diff>

<commit_message>
Tràmits urbanístics: informe de compatibilitat i obres; pas 3 enllaçat a la seu
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012ateu6UxL7MVs9JrFhHhY1
</commit_message>
<xml_diff>
--- a/dades.xlsx
+++ b/dades.xlsx
@@ -488,7 +488,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="B1:B31"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
     <col width="110" customWidth="1" min="2" max="2"/>
@@ -695,7 +695,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:C9"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
     <col width="16" customWidth="1" min="2" max="2"/>
@@ -872,7 +872,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:B9"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
     <col width="70" customWidth="1" min="2" max="2"/>
@@ -998,7 +998,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:C10"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
     <col width="46" customWidth="1" min="2" max="2"/>
@@ -1170,7 +1170,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:D5"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
     <col width="32" customWidth="1" min="2" max="2"/>
@@ -1305,7 +1305,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:F47"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
     <col width="26" customWidth="1" min="2" max="2"/>
@@ -1756,7 +1756,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:AB25"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
     <col width="10" customWidth="1" min="2" max="2"/>
@@ -2134,10 +2134,13 @@
       </c>
       <c r="R3" s="4" t="inlineStr">
         <is>
-          <t>Botiga, oficina, despatx o taller: declaració responsable o comunicació d'activitat | https://lalqueriadasnar.sedelectronica.es/catalog/t/df2d1685-af1d-454c-90dd-f0d077868573
+          <t>Primer pas: certificat o informe de compatibilitat urbanística | https://lalqueriadasnar.sedelectronica.es/catalog/t/e247f7c3-b1ff-42ef-8b7d-5195c14e9bbf
+Botiga, oficina, despatx o taller: declaració responsable o comunicació d'activitat | https://lalqueriadasnar.sedelectronica.es/catalog/t/df2d1685-af1d-454c-90dd-f0d077868573
 Bar, cafeteria o restaurant: declaració responsable d'establiments públics | https://lalqueriadasnar.sedelectronica.es/catalog/t/36fa4d83-67b8-4671-808c-09185dae1c62
 Activitat amb més impacte ambiental: sol·licitud de llicència d'activitat | https://lalqueriadasnar.sedelectronica.es/catalog/t/bf5e9be9-4ba9-4bbd-86cd-2f915f8b3c78
 Establiment públic que requereix llicència | https://lalqueriadasnar.sedelectronica.es/catalog/t/87679048-b42c-47a7-8c33-3d54d162f988
+Obres menors per a adequar el local: declaració responsable urbanística | https://lalqueriadasnar.sedelectronica.es/catalog/t/ef446499-fcee-4092-93ba-ffc7a8d90d1c
+Obres de més entitat: llicència urbanística | https://lalqueriadasnar.sedelectronica.es/catalog/t/15fabacb-83b1-47d1-b435-508245672051
 Ordenances municipals | https://www.lalqueriadasnar.es/el-ayuntamiento/ordenanzas-y-actas-de-plenos/</t>
         </is>
       </c>
@@ -4463,7 +4466,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:E24"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
     <col width="46" customWidth="1" min="2" max="2"/>
@@ -4956,7 +4959,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:F5"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
     <col width="20" customWidth="1" min="2" max="2"/>
@@ -5143,7 +5146,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:H11"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
     <col width="20" customWidth="1" min="2" max="2"/>
@@ -5549,7 +5552,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:D7"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
     <col width="56" customWidth="1" min="2" max="2"/>
@@ -5728,7 +5731,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:A4"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
   </cols>
@@ -5773,7 +5776,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:G6"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
     <col width="18" customWidth="1" min="2" max="2"/>
@@ -5918,12 +5921,12 @@
       </c>
       <c r="E4" s="4" t="inlineStr">
         <is>
-          <t>Com es demana</t>
+          <t>Sol·licita l'informe</t>
         </is>
       </c>
       <c r="F4" s="4" t="inlineStr">
         <is>
-          <t>fitxa.html?id=tramits-activitat</t>
+          <t>https://lalqueriadasnar.sedelectronica.es/catalog/t/e247f7c3-b1ff-42ef-8b7d-5195c14e9bbf</t>
         </is>
       </c>
       <c r="G4" s="4" t="inlineStr">

</xml_diff>

<commit_message>
Bons de consum segons les bases; expedient del Bar La Llar; enllaços a la instància general
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012ateu6UxL7MVs9JrFhHhY1
</commit_message>
<xml_diff>
--- a/dades.xlsx
+++ b/dades.xlsx
@@ -488,7 +488,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="B1:B31"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
     <col width="110" customWidth="1" min="2" max="2"/>
@@ -695,7 +695,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:C9"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
     <col width="16" customWidth="1" min="2" max="2"/>
@@ -872,7 +872,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:B9"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
     <col width="70" customWidth="1" min="2" max="2"/>
@@ -998,7 +998,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:C10"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
     <col width="46" customWidth="1" min="2" max="2"/>
@@ -1170,7 +1170,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:D5"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
     <col width="32" customWidth="1" min="2" max="2"/>
@@ -1305,7 +1305,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:F47"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
     <col width="26" customWidth="1" min="2" max="2"/>
@@ -1756,7 +1756,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:AB25"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
     <col width="10" customWidth="1" min="2" max="2"/>
@@ -2011,7 +2011,11 @@
           <t>https://www.lalqueriadasnar.es</t>
         </is>
       </c>
-      <c r="R2" s="4" t="inlineStr"/>
+      <c r="R2" s="4" t="inlineStr">
+        <is>
+          <t>Instància general (seu electrònica) | https://lalqueriadasnar.sedelectronica.es/catalog/t/5161fa8d-970e-4b48-a506-b2ac34ceafe5</t>
+        </is>
+      </c>
       <c r="S2" s="4" t="n">
         <v>38.7724</v>
       </c>
@@ -2248,7 +2252,11 @@
           <t>https://lalqueriadasnar.sedelectronica.es</t>
         </is>
       </c>
-      <c r="R4" s="4" t="inlineStr"/>
+      <c r="R4" s="4" t="inlineStr">
+        <is>
+          <t>Instància general (seu electrònica) | https://lalqueriadasnar.sedelectronica.es/catalog/t/5161fa8d-970e-4b48-a506-b2ac34ceafe5</t>
+        </is>
+      </c>
       <c r="S4" s="4" t="n"/>
       <c r="T4" s="4" t="n"/>
       <c r="U4" s="4" t="inlineStr">
@@ -2412,31 +2420,33 @@
       <c r="E6" s="4" t="inlineStr"/>
       <c r="F6" s="4" t="inlineStr">
         <is>
-          <t>Campanya municipal de 30.009 € per a impulsar la compra en el comerç local. Bons vàlids fins al 30 de desembre.</t>
+          <t>1.500 bons de 20 € per a comprar al comerç local. Es poden descarregar fins al 30 de desembre de 2026 o fins que s'esgoten.</t>
         </is>
       </c>
       <c r="G6" s="4" t="inlineStr">
         <is>
-          <t>Campanya de l'Ajuntament per a fomentar el consum en els establiments del municipi (convocatòria BDNS 933629).</t>
+          <t>Campanya «Bono-Consum L'Alqueria d'Asnar 2026», de 30.009 €, finançada íntegrament per la Diputació d'Alacant. Les persones empadronades descarreguen bons de descompte i els gasten en els comerços adherits, que cobren el descompte de l'Ajuntament.</t>
         </is>
       </c>
       <c r="H6" s="4" t="inlineStr">
         <is>
-          <t>Comerços i establiments que complisquen les condicions de les bases, i veïnat.</t>
+          <t>Comerços i empreses amb establiment obert al públic a l'Alqueria d'Asnar (per a adherir-se) i persones majors de 18 anys empadronades al municipi (per a usar els bons).</t>
         </is>
       </c>
       <c r="I6" s="4" t="inlineStr"/>
       <c r="J6" s="4" t="inlineStr">
         <is>
-          <t>Import aprovat: 30.009 €
-Adhesió de comerços: 10 dies hàbils des de la publicació al BOP
-Ús dels bons: del 15 d'octubre al 30 de desembre de 2026, o fins a esgotar-los
-Convocatòria a la Base de Dades Nacional de Subvencions: BDNS 933629</t>
+          <t>1.500 bons de 20 €; màxim 3 per persona en la primera fase
+Compra mínima: 40 € amb 1 bo, 80 € amb 2 i 120 € amb 3
+Fase 1: del 15 d'octubre a l'1 de desembre de 2026. Fase 2: del 2 al 30 de desembre, amb 3 bons més per persona si en queden
+Descàrrega a bonos.lalqueriadasnar.es o presencialment a l'Ajuntament (dimarts i dijous, de 10 a 14 h) per a majors de 65 anys o persones amb dificultats digitals
+Comerços: adhesió en 10 dies hàbils des de la publicació al BOP, per la seu electrònica (Annex I). Cal establiment permanent al municipi i estar al corrent amb l'AEAT, la Seguretat Social i l'Ajuntament
+Exclosos: estancs, supermercats de 400 m² o més, gasolineres i venda de vehicles, venda ambulant i en línia, joc i apostes, i medicaments de preu regulat</t>
         </is>
       </c>
       <c r="K6" s="4" t="inlineStr">
         <is>
-          <t>Al web de la campanya o a l'Ajuntament.</t>
+          <t>Persones: registre a bonos.lalqueriadasnar.es. Comerços: sol·licitud d'adhesió a la seu electrònica. L'Ajuntament publicarà la llista de comerços adherits.</t>
         </is>
       </c>
       <c r="L6" s="4" t="inlineStr">
@@ -2481,12 +2491,12 @@
       </c>
       <c r="X6" s="4" t="inlineStr">
         <is>
-          <t>Pendent: data de publicació al BOP</t>
+          <t>Pendent: data del BOP i comerços adherits</t>
         </is>
       </c>
       <c r="Y6" s="4" t="inlineStr">
         <is>
-          <t>Tauler de la seu electrònica, setembre i octubre de 2026 [F16]; BDNS 933629.</t>
+          <t>Bases reguladores del Bono-Consum L'Alqueria d'Asnar 2026 (Ajuntament); Convocatòria Bono-Consum 2026 de la Diputació d'Alacant, BOP núm. 137, 23/07/2026; BDNS 933629.</t>
         </is>
       </c>
       <c r="Z6" s="4" t="inlineStr">
@@ -3584,7 +3594,7 @@
       </c>
       <c r="I17" s="4" t="inlineStr">
         <is>
-          <t>Al setembre de 2026 l'Ajuntament va convocar un procediment públic per a adjudicar-ne l'explotació
+          <t>El 2 de setembre de 2026 l'Ajuntament va publicar la licitació (expedient 201/2026, procediment obert simplificat)
 La licitació va quedar deserta el 30 de setembre de 2026, després de la renúncia de l'única candidatura
 L'Ajuntament ha acordat iniciar un nou procediment. A 22 d'octubre de 2026 encara no s'ha publicat la nova convocatòria</t>
         </is>
@@ -3626,7 +3636,12 @@
           <t>https://lalqueriadasnar.sedelectronica.es</t>
         </is>
       </c>
-      <c r="R17" s="4" t="inlineStr"/>
+      <c r="R17" s="4" t="inlineStr">
+        <is>
+          <t>Expedient 201/2026: anunci de licitació | https://lalqueriadasnar.sedelectronica.es/?x=5nFB24BdL5Gg9wu3wwOF3J8lE7g936IEQ*Z18pxFC1KokMiik4C9YqBhfCIecFx2obSJwOMbVNAZNmLdBUj73A
+Plec de clàusules econòmiques i administratives | https://lalqueriadasnar.sedelectronica.es/?x=5nFB24BdL5Gg9wu3wwOF3J8lE7g936IEqRBPcsJ4QXvhIRbnyEo157wsEAXRMD-BdeWAvr3idgFo2uFd9K5r4A</t>
+        </is>
+      </c>
       <c r="S17" s="4" t="n">
         <v>38.77234</v>
       </c>
@@ -3713,7 +3728,7 @@
       </c>
       <c r="K18" s="4" t="inlineStr">
         <is>
-          <t>Tria «Oferir un local o espai» al formulari de contacte.</t>
+          <t>Comunica-ho amb el formulari de contacte (opció «Oferir un local o espai») o presenta una instància general a l'Ajuntament.</t>
         </is>
       </c>
       <c r="L18" s="4" t="inlineStr">
@@ -3726,7 +3741,11 @@
       <c r="O18" s="4" t="inlineStr"/>
       <c r="P18" s="4" t="inlineStr"/>
       <c r="Q18" s="4" t="inlineStr"/>
-      <c r="R18" s="4" t="inlineStr"/>
+      <c r="R18" s="4" t="inlineStr">
+        <is>
+          <t>Instància general (seu electrònica) | https://lalqueriadasnar.sedelectronica.es/catalog/t/5161fa8d-970e-4b48-a506-b2ac34ceafe5</t>
+        </is>
+      </c>
       <c r="S18" s="4" t="n"/>
       <c r="T18" s="4" t="n"/>
       <c r="U18" s="4" t="inlineStr">
@@ -4466,7 +4485,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:E24"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
     <col width="46" customWidth="1" min="2" max="2"/>
@@ -4959,7 +4978,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:F5"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
     <col width="20" customWidth="1" min="2" max="2"/>
@@ -5146,7 +5165,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:H11"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
     <col width="20" customWidth="1" min="2" max="2"/>
@@ -5552,7 +5571,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:D7"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
     <col width="56" customWidth="1" min="2" max="2"/>
@@ -5731,7 +5750,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:A4"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
   </cols>
@@ -5776,7 +5795,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:G6"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
     <col width="18" customWidth="1" min="2" max="2"/>

</xml_diff>

<commit_message>
Bons de consum: es presenta com a campanya de consum local a Oportunitats
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012ateu6UxL7MVs9JrFhHhY1
</commit_message>
<xml_diff>
--- a/dades.xlsx
+++ b/dades.xlsx
@@ -2409,28 +2409,32 @@
       </c>
       <c r="C6" s="4" t="inlineStr">
         <is>
-          <t>municipal</t>
+          <t>oportunitat</t>
         </is>
       </c>
       <c r="D6" s="4" t="inlineStr">
         <is>
-          <t>Bons de consum local 2026</t>
-        </is>
-      </c>
-      <c r="E6" s="4" t="inlineStr"/>
+          <t>Campanya de consum local (Bono-Consum 2026)</t>
+        </is>
+      </c>
+      <c r="E6" s="4" t="inlineStr">
+        <is>
+          <t>Campanya 2026 en curs, fins al 30 de desembre</t>
+        </is>
+      </c>
       <c r="F6" s="4" t="inlineStr">
         <is>
-          <t>1.500 bons de 20 € per a comprar al comerç local. Es poden descarregar fins al 30 de desembre de 2026 o fins que s'esgoten.</t>
+          <t>L'Ajuntament impulsa el comerç local amb una campanya de bons de descompte per als veïns. Els comerços del poble s'hi poden adherir a cada edició.</t>
         </is>
       </c>
       <c r="G6" s="4" t="inlineStr">
         <is>
-          <t>Campanya «Bono-Consum L'Alqueria d'Asnar 2026», de 30.009 €, finançada íntegrament per la Diputació d'Alacant. Les persones empadronades descarreguen bons de descompte i els gasten en els comerços adherits, que cobren el descompte de l'Ajuntament.</t>
+          <t>Campanya «Bono-Consum L'Alqueria d'Asnar 2026», de 30.009 €, finançada íntegrament per la Diputació d'Alacant. Les persones empadronades descarreguen bons de descompte i els gasten en els comerços adherits, que cobren el descompte de l'Ajuntament. És una mostra del suport municipal al comerç de proximitat: els comerços que obrin al municipi podran adherir-se a les properes edicions.</t>
         </is>
       </c>
       <c r="H6" s="4" t="inlineStr">
         <is>
-          <t>Comerços i empreses amb establiment obert al públic a l'Alqueria d'Asnar (per a adherir-se) i persones majors de 18 anys empadronades al municipi (per a usar els bons).</t>
+          <t>Comerços i establiments oberts al públic al municipi, que s'hi poden adherir, i persones majors de 18 anys empadronades, que usen els bons.</t>
         </is>
       </c>
       <c r="I6" s="4" t="inlineStr"/>
@@ -2446,7 +2450,7 @@
       </c>
       <c r="K6" s="4" t="inlineStr">
         <is>
-          <t>Persones: registre a bonos.lalqueriadasnar.es. Comerços: sol·licitud d'adhesió a la seu electrònica. L'Ajuntament publicarà la llista de comerços adherits.</t>
+          <t>Comerços: l'adhesió s'obri a cada edició durant 10 dies hàbils des de la publicació de la convocatòria al BOP, per la seu electrònica. Persones: registre a bonos.lalqueriadasnar.es.</t>
         </is>
       </c>
       <c r="L6" s="4" t="inlineStr">
@@ -2481,7 +2485,7 @@
       </c>
       <c r="V6" s="4" t="inlineStr">
         <is>
-          <t>sí</t>
+          <t>no</t>
         </is>
       </c>
       <c r="W6" s="4" t="inlineStr">
@@ -5481,7 +5485,7 @@
       </c>
       <c r="F9" s="4" t="inlineStr">
         <is>
-          <t>bons-consum-2026, labora, ivace</t>
+          <t>labora, ivace</t>
         </is>
       </c>
       <c r="G9" s="4" t="inlineStr"/>
@@ -5500,10 +5504,14 @@
       </c>
       <c r="C10" s="4" t="inlineStr">
         <is>
-          <t>Necessitat detectada per l'Ajuntament</t>
-        </is>
-      </c>
-      <c r="D10" s="4" t="inlineStr"/>
+          <t>Hostaleria i comerç de proximitat</t>
+        </is>
+      </c>
+      <c r="D10" s="4" t="inlineStr">
+        <is>
+          <t>Necessitat detectada per l'Ajuntament i suport municipal al comerç local.</t>
+        </is>
+      </c>
       <c r="E10" s="4" t="inlineStr">
         <is>
           <t>foto</t>
@@ -5511,7 +5519,7 @@
       </c>
       <c r="F10" s="4" t="inlineStr">
         <is>
-          <t>op-proximitat, bar-la-llar</t>
+          <t>op-proximitat, bar-la-llar, bons-consum-2026</t>
         </is>
       </c>
       <c r="G10" s="4" t="inlineStr"/>
@@ -6024,7 +6032,7 @@
       </c>
       <c r="G6" s="4" t="inlineStr">
         <is>
-          <t>labora, ivace, bons-consum-2026</t>
+          <t>labora, ivace</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Horari d'atenció de l'Ajuntament: de 9.00 a 14.00 h
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012ateu6UxL7MVs9JrFhHhY1
</commit_message>
<xml_diff>
--- a/dades.xlsx
+++ b/dades.xlsx
@@ -946,7 +946,7 @@
       </c>
       <c r="B6" s="4" t="inlineStr">
         <is>
-          <t>Dilluns a divendres, de 8.00 a 14.30 h</t>
+          <t>Dilluns a divendres, de 9.00 a 14.00 h</t>
         </is>
       </c>
     </row>
@@ -2003,7 +2003,7 @@
       </c>
       <c r="P2" s="4" t="inlineStr">
         <is>
-          <t>Dilluns a divendres, de 8.00 a 14.30 h</t>
+          <t>Dilluns a divendres, de 9.00 a 14.00 h</t>
         </is>
       </c>
       <c r="Q2" s="4" t="inlineStr">
@@ -2034,17 +2034,13 @@
       </c>
       <c r="W2" s="4" t="inlineStr">
         <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="X2" s="4" t="inlineStr">
-        <is>
-          <t>Pendent: confirmar horari</t>
-        </is>
-      </c>
+          <t>sí</t>
+        </is>
+      </c>
+      <c r="X2" s="4" t="inlineStr"/>
       <c r="Y2" s="4" t="inlineStr">
         <is>
-          <t>Registre d'Entitats Locals GVA [F01]; web municipal. Horari pendent de confirmació oficial.</t>
+          <t>Registre d'Entitats Locals GVA [F01]; seu electrònica municipal (horari d'atenció al públic, 26/10/2026).</t>
         </is>
       </c>
       <c r="Z2" s="4" t="inlineStr">

</xml_diff>